<commit_message>
Atualização automática - 17/06/2026 15:21
</commit_message>
<xml_diff>
--- a/Aplicativos/import_querys/divergencias_venda_maio.xlsx
+++ b/Aplicativos/import_querys/divergencias_venda_maio.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -706,9 +706,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Escritório">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -746,7 +746,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Escritório">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -816,7 +816,7 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Escritório">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -992,17 +992,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J201"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="56.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="40" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
@@ -1053,13 +1042,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>160569.04999999999</v>
+        <v>160569.05</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>-160569.04999999999</v>
+        <v>-160569.05</v>
       </c>
       <c r="J2" t="s">
         <v>212</v>
@@ -1076,7 +1065,7 @@
         <v>800</v>
       </c>
       <c r="E3">
-        <v>5790.6970000000001</v>
+        <v>5790.697</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -1134,19 +1123,19 @@
         <v>800</v>
       </c>
       <c r="E5">
-        <v>52.133000000000003</v>
+        <v>52.133</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>2462.7399999999998</v>
+        <v>2462.74</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5">
-        <v>-2462.7399999999998</v>
+        <v>-2462.74</v>
       </c>
       <c r="J5" t="s">
         <v>212</v>
@@ -1201,10 +1190,10 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>563.05999999999995</v>
+        <v>563.0599999999999</v>
       </c>
       <c r="I7">
-        <v>563.05999999999995</v>
+        <v>563.0599999999999</v>
       </c>
       <c r="J7" t="s">
         <v>213</v>
@@ -1230,10 +1219,10 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>557.07000000000005</v>
+        <v>557.0700000000001</v>
       </c>
       <c r="I8">
-        <v>557.07000000000005</v>
+        <v>557.0700000000001</v>
       </c>
       <c r="J8" t="s">
         <v>213</v>
@@ -1375,10 +1364,10 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>135.83000000000001</v>
+        <v>135.83</v>
       </c>
       <c r="I13">
-        <v>135.83000000000001</v>
+        <v>135.83</v>
       </c>
       <c r="J13" t="s">
         <v>213</v>
@@ -1926,10 +1915,10 @@
         <v>0</v>
       </c>
       <c r="H32">
-        <v>33.979999999999997</v>
+        <v>33.98</v>
       </c>
       <c r="I32">
-        <v>33.979999999999997</v>
+        <v>33.98</v>
       </c>
       <c r="J32" t="s">
         <v>213</v>
@@ -1978,10 +1967,10 @@
         <v>800</v>
       </c>
       <c r="E34">
-        <v>706.78300000000002</v>
+        <v>706.783</v>
       </c>
       <c r="F34">
-        <v>706.78300000000002</v>
+        <v>706.783</v>
       </c>
       <c r="G34">
         <v>22780.16</v>
@@ -1990,7 +1979,7 @@
         <v>22762.67</v>
       </c>
       <c r="I34">
-        <v>-17.490000000001601</v>
+        <v>-17.4900000000016</v>
       </c>
       <c r="J34" t="s">
         <v>214</v>
@@ -2167,7 +2156,7 @@
         <v>779291.22</v>
       </c>
       <c r="I40">
-        <v>-4.1099999999860302</v>
+        <v>-4.10999999998603</v>
       </c>
       <c r="J40" t="s">
         <v>214</v>
@@ -2196,10 +2185,10 @@
         <v>89794.28</v>
       </c>
       <c r="H41">
-        <v>89790.57</v>
+        <v>89790.57000000001</v>
       </c>
       <c r="I41">
-        <v>-3.7099999999918509</v>
+        <v>-3.709999999991851</v>
       </c>
       <c r="J41" t="s">
         <v>214</v>
@@ -2228,10 +2217,10 @@
         <v>90986.86</v>
       </c>
       <c r="H42">
-        <v>90983.26</v>
+        <v>90983.25999999999</v>
       </c>
       <c r="I42">
-        <v>-3.6000000000058212</v>
+        <v>-3.600000000005821</v>
       </c>
       <c r="J42" t="s">
         <v>214</v>
@@ -2280,13 +2269,13 @@
         <v>800</v>
       </c>
       <c r="E44">
-        <v>73977.210999999996</v>
+        <v>73977.211</v>
       </c>
       <c r="F44">
-        <v>73977.210999999996</v>
+        <v>73977.211</v>
       </c>
       <c r="G44">
-        <v>594276.30000000005</v>
+        <v>594276.3</v>
       </c>
       <c r="H44">
         <v>594273.61</v>
@@ -2321,10 +2310,10 @@
         <v>590762</v>
       </c>
       <c r="H45">
-        <v>590759.56999999995</v>
+        <v>590759.5699999999</v>
       </c>
       <c r="I45">
-        <v>-2.4300000000512232</v>
+        <v>-2.430000000051223</v>
       </c>
       <c r="J45" t="s">
         <v>214</v>
@@ -2350,13 +2339,13 @@
         <v>5739</v>
       </c>
       <c r="G46">
-        <v>90412.76</v>
+        <v>90412.75999999999</v>
       </c>
       <c r="H46">
         <v>90410.61</v>
       </c>
       <c r="I46">
-        <v>-2.1499999999941788</v>
+        <v>-2.149999999994179</v>
       </c>
       <c r="J46" t="s">
         <v>214</v>
@@ -2376,16 +2365,16 @@
         <v>800</v>
       </c>
       <c r="E47">
-        <v>64498.682000000001</v>
+        <v>64498.682</v>
       </c>
       <c r="F47">
-        <v>64498.682000000001</v>
+        <v>64498.682</v>
       </c>
       <c r="G47">
         <v>632252.76</v>
       </c>
       <c r="H47">
-        <v>632250.82999999996</v>
+        <v>632250.83</v>
       </c>
       <c r="I47">
         <v>-1.930000000051223</v>
@@ -2414,13 +2403,13 @@
         <v>54722</v>
       </c>
       <c r="G48">
-        <v>1190656.0900000001</v>
+        <v>1190656.09</v>
       </c>
       <c r="H48">
         <v>1190654.44</v>
       </c>
       <c r="I48">
-        <v>-1.6500000001396979</v>
+        <v>-1.650000000139698</v>
       </c>
       <c r="J48" t="s">
         <v>214</v>
@@ -2472,10 +2461,10 @@
         <v>800</v>
       </c>
       <c r="E50">
-        <v>21484.207999999999</v>
+        <v>21484.208</v>
       </c>
       <c r="F50">
-        <v>21484.207999999999</v>
+        <v>21484.208</v>
       </c>
       <c r="G50">
         <v>557504.03</v>
@@ -2484,7 +2473,7 @@
         <v>557502.87</v>
       </c>
       <c r="I50">
-        <v>-1.1600000000325961</v>
+        <v>-1.160000000032596</v>
       </c>
       <c r="J50" t="s">
         <v>214</v>
@@ -2548,7 +2537,7 @@
         <v>1467.83</v>
       </c>
       <c r="I52">
-        <v>-1.0800000000001551</v>
+        <v>-1.080000000000155</v>
       </c>
       <c r="J52" t="s">
         <v>214</v>
@@ -2577,10 +2566,10 @@
         <v>4837.87</v>
       </c>
       <c r="H53">
-        <v>4836.8900000000003</v>
+        <v>4836.89</v>
       </c>
       <c r="I53">
-        <v>-0.97999999999956344</v>
+        <v>-0.9799999999995634</v>
       </c>
       <c r="J53" t="s">
         <v>214</v>
@@ -2606,13 +2595,13 @@
         <v>7403.433</v>
       </c>
       <c r="G54">
-        <v>264866.71000000002</v>
+        <v>264866.71</v>
       </c>
       <c r="H54">
-        <v>264865.78000000003</v>
+        <v>264865.78</v>
       </c>
       <c r="I54">
-        <v>-0.92999999999301508</v>
+        <v>-0.9299999999930151</v>
       </c>
       <c r="J54" t="s">
         <v>214</v>
@@ -2632,10 +2621,10 @@
         <v>800</v>
       </c>
       <c r="E55">
-        <v>4149.3509999999997</v>
+        <v>4149.351</v>
       </c>
       <c r="F55">
-        <v>4149.3509999999997</v>
+        <v>4149.351</v>
       </c>
       <c r="G55">
         <v>178491.71</v>
@@ -2644,7 +2633,7 @@
         <v>178490.8</v>
       </c>
       <c r="I55">
-        <v>-0.91000000000349246</v>
+        <v>-0.9100000000034925</v>
       </c>
       <c r="J55" t="s">
         <v>214</v>
@@ -2664,10 +2653,10 @@
         <v>800</v>
       </c>
       <c r="E56">
-        <v>23022.567999999999</v>
+        <v>23022.568</v>
       </c>
       <c r="F56">
-        <v>23022.567999999999</v>
+        <v>23022.568</v>
       </c>
       <c r="G56">
         <v>1014650.43</v>
@@ -2676,7 +2665,7 @@
         <v>1014649.55</v>
       </c>
       <c r="I56">
-        <v>-0.88000000000465661</v>
+        <v>-0.8800000000046566</v>
       </c>
       <c r="J56" t="s">
         <v>214</v>
@@ -2708,7 +2697,7 @@
         <v>110994.96</v>
       </c>
       <c r="I57">
-        <v>-0.83999999999650754</v>
+        <v>-0.8399999999965075</v>
       </c>
       <c r="J57" t="s">
         <v>214</v>
@@ -2728,10 +2717,10 @@
         <v>800</v>
       </c>
       <c r="E58">
-        <v>17973.719000000001</v>
+        <v>17973.719</v>
       </c>
       <c r="F58">
-        <v>17973.719000000001</v>
+        <v>17973.719</v>
       </c>
       <c r="G58">
         <v>190017.87</v>
@@ -2740,7 +2729,7 @@
         <v>190017.06</v>
       </c>
       <c r="I58">
-        <v>-0.80999999999767169</v>
+        <v>-0.8099999999976717</v>
       </c>
       <c r="J58" t="s">
         <v>214</v>
@@ -2792,10 +2781,10 @@
         <v>800</v>
       </c>
       <c r="E60">
-        <v>1737.5429999999999</v>
+        <v>1737.543</v>
       </c>
       <c r="F60">
-        <v>1737.5429999999999</v>
+        <v>1737.543</v>
       </c>
       <c r="G60">
         <v>22295.14</v>
@@ -2804,7 +2793,7 @@
         <v>22294.36</v>
       </c>
       <c r="I60">
-        <v>-0.77999999999883585</v>
+        <v>-0.7799999999988358</v>
       </c>
       <c r="J60" t="s">
         <v>214</v>
@@ -2824,10 +2813,10 @@
         <v>800</v>
       </c>
       <c r="E61">
-        <v>37561.732000000004</v>
+        <v>37561.732</v>
       </c>
       <c r="F61">
-        <v>37561.732000000004</v>
+        <v>37561.732</v>
       </c>
       <c r="G61">
         <v>412254.86</v>
@@ -2836,7 +2825,7 @@
         <v>412254.09</v>
       </c>
       <c r="I61">
-        <v>-0.76999999996041879</v>
+        <v>-0.7699999999604188</v>
       </c>
       <c r="J61" t="s">
         <v>214</v>
@@ -2868,7 +2857,7 @@
         <v>135672.99</v>
       </c>
       <c r="I62">
-        <v>-0.76000000000931323</v>
+        <v>-0.7600000000093132</v>
       </c>
       <c r="J62" t="s">
         <v>214</v>
@@ -2888,10 +2877,10 @@
         <v>800</v>
       </c>
       <c r="E63">
-        <v>7253.1329999999998</v>
+        <v>7253.133</v>
       </c>
       <c r="F63">
-        <v>7253.1329999999998</v>
+        <v>7253.133</v>
       </c>
       <c r="G63">
         <v>159440.25</v>
@@ -2926,10 +2915,10 @@
         <v>6734</v>
       </c>
       <c r="G64">
-        <v>39592.410000000003</v>
+        <v>39592.41</v>
       </c>
       <c r="H64">
-        <v>39591.660000000003</v>
+        <v>39591.66</v>
       </c>
       <c r="I64">
         <v>-0.75</v>
@@ -2958,13 +2947,13 @@
         <v>10303.234</v>
       </c>
       <c r="G65">
-        <v>41007.440000000002</v>
+        <v>41007.44</v>
       </c>
       <c r="H65">
         <v>41006.76</v>
       </c>
       <c r="I65">
-        <v>-0.68000000000029104</v>
+        <v>-0.680000000000291</v>
       </c>
       <c r="J65" t="s">
         <v>214</v>
@@ -2996,7 +2985,7 @@
         <v>481909.65</v>
       </c>
       <c r="I66">
-        <v>-0.63000000000465661</v>
+        <v>-0.6300000000046566</v>
       </c>
       <c r="J66" t="s">
         <v>214</v>
@@ -3022,13 +3011,13 @@
         <v>1936</v>
       </c>
       <c r="G67">
-        <v>8653.64</v>
+        <v>8653.639999999999</v>
       </c>
       <c r="H67">
-        <v>8653.0400000000009</v>
+        <v>8653.040000000001</v>
       </c>
       <c r="I67">
-        <v>-0.59999999999854481</v>
+        <v>-0.5999999999985448</v>
       </c>
       <c r="J67" t="s">
         <v>214</v>
@@ -3054,13 +3043,13 @@
         <v>1769</v>
       </c>
       <c r="G68">
-        <v>10227.209999999999</v>
+        <v>10227.21</v>
       </c>
       <c r="H68">
         <v>10226.61</v>
       </c>
       <c r="I68">
-        <v>-0.59999999999854481</v>
+        <v>-0.5999999999985448</v>
       </c>
       <c r="J68" t="s">
         <v>214</v>
@@ -3086,13 +3075,13 @@
         <v>6520</v>
       </c>
       <c r="G69">
-        <v>77116.149999999994</v>
+        <v>77116.14999999999</v>
       </c>
       <c r="H69">
         <v>77115.55</v>
       </c>
       <c r="I69">
-        <v>-0.59999999999126885</v>
+        <v>-0.5999999999912689</v>
       </c>
       <c r="J69" t="s">
         <v>214</v>
@@ -3124,7 +3113,7 @@
         <v>449.19</v>
       </c>
       <c r="I70">
-        <v>-0.56999999999999318</v>
+        <v>-0.5699999999999932</v>
       </c>
       <c r="J70" t="s">
         <v>214</v>
@@ -3176,10 +3165,10 @@
         <v>800</v>
       </c>
       <c r="E72">
-        <v>8684.4529999999995</v>
+        <v>8684.453</v>
       </c>
       <c r="F72">
-        <v>8684.4529999999995</v>
+        <v>8684.453</v>
       </c>
       <c r="G72">
         <v>48574.13</v>
@@ -3188,7 +3177,7 @@
         <v>48573.59</v>
       </c>
       <c r="I72">
-        <v>-0.54000000000087311</v>
+        <v>-0.5400000000008731</v>
       </c>
       <c r="J72" t="s">
         <v>214</v>
@@ -3220,7 +3209,7 @@
         <v>69150.41</v>
       </c>
       <c r="I73">
-        <v>-0.53999999999359716</v>
+        <v>-0.5399999999935972</v>
       </c>
       <c r="J73" t="s">
         <v>214</v>
@@ -3240,10 +3229,10 @@
         <v>800</v>
       </c>
       <c r="E74">
-        <v>41.387999999999998</v>
+        <v>41.388</v>
       </c>
       <c r="F74">
-        <v>41.387999999999998</v>
+        <v>41.388</v>
       </c>
       <c r="G74">
         <v>2441.94</v>
@@ -3252,7 +3241,7 @@
         <v>2441.42</v>
       </c>
       <c r="I74">
-        <v>-0.51999999999998181</v>
+        <v>-0.5199999999999818</v>
       </c>
       <c r="J74" t="s">
         <v>214</v>
@@ -3284,7 +3273,7 @@
         <v>51883.54</v>
       </c>
       <c r="I75">
-        <v>-0.51999999999679858</v>
+        <v>-0.5199999999967986</v>
       </c>
       <c r="J75" t="s">
         <v>214</v>
@@ -3316,7 +3305,7 @@
         <v>2681.31</v>
       </c>
       <c r="I76">
-        <v>-0.51000000000021828</v>
+        <v>-0.5100000000002183</v>
       </c>
       <c r="J76" t="s">
         <v>214</v>
@@ -3348,7 +3337,7 @@
         <v>11512.23</v>
       </c>
       <c r="I77">
-        <v>-0.51000000000021828</v>
+        <v>-0.5100000000002183</v>
       </c>
       <c r="J77" t="s">
         <v>214</v>
@@ -3380,7 +3369,7 @@
         <v>11217.03</v>
       </c>
       <c r="I78">
-        <v>-0.48999999999978172</v>
+        <v>-0.4899999999997817</v>
       </c>
       <c r="J78" t="s">
         <v>214</v>
@@ -3412,7 +3401,7 @@
         <v>7113.19</v>
       </c>
       <c r="I79">
-        <v>-0.48000000000047288</v>
+        <v>-0.4800000000004729</v>
       </c>
       <c r="J79" t="s">
         <v>214</v>
@@ -3432,19 +3421,19 @@
         <v>800</v>
       </c>
       <c r="E80">
-        <v>76919.672000000006</v>
+        <v>76919.67200000001</v>
       </c>
       <c r="F80">
-        <v>76919.672000000006</v>
+        <v>76919.67200000001</v>
       </c>
       <c r="G80">
-        <v>298431.65000000002</v>
+        <v>298431.65</v>
       </c>
       <c r="H80">
         <v>298431.18</v>
       </c>
       <c r="I80">
-        <v>-0.47000000003026798</v>
+        <v>-0.470000000030268</v>
       </c>
       <c r="J80" t="s">
         <v>214</v>
@@ -3464,10 +3453,10 @@
         <v>800</v>
       </c>
       <c r="E81">
-        <v>24356.521000000001</v>
+        <v>24356.521</v>
       </c>
       <c r="F81">
-        <v>24356.521000000001</v>
+        <v>24356.521</v>
       </c>
       <c r="G81">
         <v>118440.62</v>
@@ -3476,7 +3465,7 @@
         <v>118440.16</v>
       </c>
       <c r="I81">
-        <v>-0.45999999999185093</v>
+        <v>-0.4599999999918509</v>
       </c>
       <c r="J81" t="s">
         <v>214</v>
@@ -3537,10 +3526,10 @@
         <v>69325.02</v>
       </c>
       <c r="H83">
-        <v>69324.570000000007</v>
+        <v>69324.57000000001</v>
       </c>
       <c r="I83">
-        <v>-0.44999999999708962</v>
+        <v>-0.4499999999970896</v>
       </c>
       <c r="J83" t="s">
         <v>214</v>
@@ -3569,10 +3558,10 @@
         <v>74413.66</v>
       </c>
       <c r="H84">
-        <v>74413.210000000006</v>
+        <v>74413.21000000001</v>
       </c>
       <c r="I84">
-        <v>-0.44999999999708962</v>
+        <v>-0.4499999999970896</v>
       </c>
       <c r="J84" t="s">
         <v>214</v>
@@ -3604,7 +3593,7 @@
         <v>14337.57</v>
       </c>
       <c r="I85">
-        <v>-0.43000000000029098</v>
+        <v>-0.430000000000291</v>
       </c>
       <c r="J85" t="s">
         <v>214</v>
@@ -3636,7 +3625,7 @@
         <v>23751.54</v>
       </c>
       <c r="I86">
-        <v>-0.41999999999825383</v>
+        <v>-0.4199999999982538</v>
       </c>
       <c r="J86" t="s">
         <v>214</v>
@@ -3668,7 +3657,7 @@
         <v>53784.44</v>
       </c>
       <c r="I87">
-        <v>-0.39999999999417918</v>
+        <v>-0.3999999999941792</v>
       </c>
       <c r="J87" t="s">
         <v>214</v>
@@ -3700,7 +3689,7 @@
         <v>408590.14</v>
       </c>
       <c r="I88">
-        <v>-0.39000000001396978</v>
+        <v>-0.3900000000139698</v>
       </c>
       <c r="J88" t="s">
         <v>214</v>
@@ -3720,10 +3709,10 @@
         <v>800</v>
       </c>
       <c r="E89">
-        <v>10635.199000000001</v>
+        <v>10635.199</v>
       </c>
       <c r="F89">
-        <v>10635.199000000001</v>
+        <v>10635.199</v>
       </c>
       <c r="G89">
         <v>104935.29</v>
@@ -3732,7 +3721,7 @@
         <v>104934.9</v>
       </c>
       <c r="I89">
-        <v>-0.38999999999941792</v>
+        <v>-0.3899999999994179</v>
       </c>
       <c r="J89" t="s">
         <v>214</v>
@@ -3758,13 +3747,13 @@
         <v>8109</v>
       </c>
       <c r="G90">
-        <v>40090.300000000003</v>
+        <v>40090.3</v>
       </c>
       <c r="H90">
-        <v>40089.910000000003</v>
+        <v>40089.91</v>
       </c>
       <c r="I90">
-        <v>-0.38999999999941792</v>
+        <v>-0.3899999999994179</v>
       </c>
       <c r="J90" t="s">
         <v>214</v>
@@ -3796,7 +3785,7 @@
         <v>74049.84</v>
       </c>
       <c r="I91">
-        <v>-0.38999999999941792</v>
+        <v>-0.3899999999994179</v>
       </c>
       <c r="J91" t="s">
         <v>214</v>
@@ -3828,7 +3817,7 @@
         <v>50051.59</v>
       </c>
       <c r="I92">
-        <v>-0.38000000000465661</v>
+        <v>-0.3800000000046566</v>
       </c>
       <c r="J92" t="s">
         <v>214</v>
@@ -3860,7 +3849,7 @@
         <v>66997.42</v>
       </c>
       <c r="I93">
-        <v>-0.38000000000465661</v>
+        <v>-0.3800000000046566</v>
       </c>
       <c r="J93" t="s">
         <v>214</v>
@@ -3892,7 +3881,7 @@
         <v>12277.47</v>
       </c>
       <c r="I94">
-        <v>-0.38000000000101858</v>
+        <v>-0.3800000000010186</v>
       </c>
       <c r="J94" t="s">
         <v>214</v>
@@ -3924,7 +3913,7 @@
         <v>25953.87</v>
       </c>
       <c r="I95">
-        <v>-0.38000000000101858</v>
+        <v>-0.3800000000010186</v>
       </c>
       <c r="J95" t="s">
         <v>214</v>
@@ -3956,7 +3945,7 @@
         <v>13.99</v>
       </c>
       <c r="I96">
-        <v>-0.36999999999999922</v>
+        <v>-0.3699999999999992</v>
       </c>
       <c r="J96" t="s">
         <v>214</v>
@@ -3988,7 +3977,7 @@
         <v>5554.6</v>
       </c>
       <c r="I97">
-        <v>-0.36999999999989092</v>
+        <v>-0.3699999999998909</v>
       </c>
       <c r="J97" t="s">
         <v>214</v>
@@ -4017,10 +4006,10 @@
         <v>1104.52</v>
       </c>
       <c r="H98">
-        <v>1104.1500000000001</v>
+        <v>1104.15</v>
       </c>
       <c r="I98">
-        <v>-0.36999999999989092</v>
+        <v>-0.3699999999998909</v>
       </c>
       <c r="J98" t="s">
         <v>214</v>
@@ -4040,19 +4029,19 @@
         <v>800</v>
       </c>
       <c r="E99">
-        <v>17009.686000000002</v>
+        <v>17009.686</v>
       </c>
       <c r="F99">
-        <v>17009.686000000002</v>
+        <v>17009.686</v>
       </c>
       <c r="G99">
         <v>166945.01</v>
       </c>
       <c r="H99">
-        <v>166944.64000000001</v>
+        <v>166944.64</v>
       </c>
       <c r="I99">
-        <v>-0.36999999999534339</v>
+        <v>-0.3699999999953434</v>
       </c>
       <c r="J99" t="s">
         <v>214</v>
@@ -4072,19 +4061,19 @@
         <v>800</v>
       </c>
       <c r="E100">
-        <v>2256.5889999999999</v>
+        <v>2256.589</v>
       </c>
       <c r="F100">
-        <v>2256.5889999999999</v>
+        <v>2256.589</v>
       </c>
       <c r="G100">
-        <v>39961.599999999999</v>
+        <v>39961.6</v>
       </c>
       <c r="H100">
         <v>39961.25</v>
       </c>
       <c r="I100">
-        <v>-0.34999999999854481</v>
+        <v>-0.3499999999985448</v>
       </c>
       <c r="J100" t="s">
         <v>214</v>
@@ -4110,13 +4099,13 @@
         <v>182</v>
       </c>
       <c r="G101">
-        <v>2225.2600000000002</v>
+        <v>2225.26</v>
       </c>
       <c r="H101">
         <v>2224.92</v>
       </c>
       <c r="I101">
-        <v>-0.34000000000014552</v>
+        <v>-0.3400000000001455</v>
       </c>
       <c r="J101" t="s">
         <v>214</v>
@@ -4148,7 +4137,7 @@
         <v>42128.77</v>
       </c>
       <c r="I102">
-        <v>-0.33000000000174617</v>
+        <v>-0.3300000000017462</v>
       </c>
       <c r="J102" t="s">
         <v>214</v>
@@ -4168,19 +4157,19 @@
         <v>800</v>
       </c>
       <c r="E103">
-        <v>8313.3580000000002</v>
+        <v>8313.358</v>
       </c>
       <c r="F103">
-        <v>8313.3580000000002</v>
+        <v>8313.358</v>
       </c>
       <c r="G103">
-        <v>88317.15</v>
+        <v>88317.14999999999</v>
       </c>
       <c r="H103">
-        <v>88316.82</v>
+        <v>88316.82000000001</v>
       </c>
       <c r="I103">
-        <v>-0.32999999998719431</v>
+        <v>-0.3299999999871943</v>
       </c>
       <c r="J103" t="s">
         <v>214</v>
@@ -4212,7 +4201,7 @@
         <v>233603.21</v>
       </c>
       <c r="I104">
-        <v>-0.32000000000698492</v>
+        <v>-0.3200000000069849</v>
       </c>
       <c r="J104" t="s">
         <v>214</v>
@@ -4244,7 +4233,7 @@
         <v>7201.95</v>
       </c>
       <c r="I105">
-        <v>-0.32000000000061851</v>
+        <v>-0.3200000000006185</v>
       </c>
       <c r="J105" t="s">
         <v>214</v>
@@ -4276,7 +4265,7 @@
         <v>18687.86</v>
       </c>
       <c r="I106">
-        <v>-0.31999999999970902</v>
+        <v>-0.319999999999709</v>
       </c>
       <c r="J106" t="s">
         <v>214</v>
@@ -4308,7 +4297,7 @@
         <v>9310.27</v>
       </c>
       <c r="I107">
-        <v>-0.31999999999970902</v>
+        <v>-0.319999999999709</v>
       </c>
       <c r="J107" t="s">
         <v>214</v>
@@ -4340,7 +4329,7 @@
         <v>4765.01</v>
       </c>
       <c r="I108">
-        <v>-0.31999999999970902</v>
+        <v>-0.319999999999709</v>
       </c>
       <c r="J108" t="s">
         <v>214</v>
@@ -4366,13 +4355,13 @@
         <v>5957</v>
       </c>
       <c r="G109">
-        <v>68446.240000000005</v>
+        <v>68446.24000000001</v>
       </c>
       <c r="H109">
-        <v>68445.929999999993</v>
+        <v>68445.92999999999</v>
       </c>
       <c r="I109">
-        <v>-0.31000000001222361</v>
+        <v>-0.3100000000122236</v>
       </c>
       <c r="J109" t="s">
         <v>214</v>
@@ -4404,7 +4393,7 @@
         <v>2143.86</v>
       </c>
       <c r="I110">
-        <v>-0.30999999999994537</v>
+        <v>-0.3099999999999454</v>
       </c>
       <c r="J110" t="s">
         <v>214</v>
@@ -4424,10 +4413,10 @@
         <v>800</v>
       </c>
       <c r="E111">
-        <v>7055.8119999999999</v>
+        <v>7055.812</v>
       </c>
       <c r="F111">
-        <v>7055.8119999999999</v>
+        <v>7055.812</v>
       </c>
       <c r="G111">
         <v>22479.51</v>
@@ -4468,7 +4457,7 @@
         <v>3772.21</v>
       </c>
       <c r="I112">
-        <v>-0.27999999999974529</v>
+        <v>-0.2799999999997453</v>
       </c>
       <c r="J112" t="s">
         <v>214</v>
@@ -4488,10 +4477,10 @@
         <v>800</v>
       </c>
       <c r="E113">
-        <v>38090.824999999997</v>
+        <v>38090.825</v>
       </c>
       <c r="F113">
-        <v>38090.824999999997</v>
+        <v>38090.825</v>
       </c>
       <c r="G113">
         <v>609079.01</v>
@@ -4500,7 +4489,7 @@
         <v>609078.74</v>
       </c>
       <c r="I113">
-        <v>-0.27000000001862651</v>
+        <v>-0.2700000000186265</v>
       </c>
       <c r="J113" t="s">
         <v>214</v>
@@ -4520,19 +4509,19 @@
         <v>800</v>
       </c>
       <c r="E114">
-        <v>32509.246999999999</v>
+        <v>32509.247</v>
       </c>
       <c r="F114">
-        <v>32509.246999999999</v>
+        <v>32509.247</v>
       </c>
       <c r="G114">
         <v>86573.45</v>
       </c>
       <c r="H114">
-        <v>86573.18</v>
+        <v>86573.17999999999</v>
       </c>
       <c r="I114">
-        <v>-0.27000000000407448</v>
+        <v>-0.2700000000040745</v>
       </c>
       <c r="J114" t="s">
         <v>214</v>
@@ -4561,10 +4550,10 @@
         <v>17125.53</v>
       </c>
       <c r="H115">
-        <v>17125.259999999998</v>
+        <v>17125.26</v>
       </c>
       <c r="I115">
-        <v>-0.27000000000043661</v>
+        <v>-0.2700000000004366</v>
       </c>
       <c r="J115" t="s">
         <v>214</v>
@@ -4596,7 +4585,7 @@
         <v>8083.98</v>
       </c>
       <c r="I116">
-        <v>-0.27000000000043661</v>
+        <v>-0.2700000000004366</v>
       </c>
       <c r="J116" t="s">
         <v>214</v>
@@ -4628,7 +4617,7 @@
         <v>1150.99</v>
       </c>
       <c r="I117">
-        <v>-0.25999999999999091</v>
+        <v>-0.2599999999999909</v>
       </c>
       <c r="J117" t="s">
         <v>214</v>
@@ -4654,13 +4643,13 @@
         <v>18341.302</v>
       </c>
       <c r="G118">
-        <v>94879.360000000001</v>
+        <v>94879.36</v>
       </c>
       <c r="H118">
-        <v>94879.1</v>
+        <v>94879.10000000001</v>
       </c>
       <c r="I118">
-        <v>-0.25999999999476131</v>
+        <v>-0.2599999999947613</v>
       </c>
       <c r="J118" t="s">
         <v>214</v>
@@ -4721,10 +4710,10 @@
         <v>17359.5</v>
       </c>
       <c r="H120">
-        <v>17359.259999999998</v>
+        <v>17359.26</v>
       </c>
       <c r="I120">
-        <v>-0.24000000000160071</v>
+        <v>-0.2400000000016007</v>
       </c>
       <c r="J120" t="s">
         <v>214</v>
@@ -4756,7 +4745,7 @@
         <v>5455.44</v>
       </c>
       <c r="I121">
-        <v>-0.24000000000069119</v>
+        <v>-0.2400000000006912</v>
       </c>
       <c r="J121" t="s">
         <v>214</v>
@@ -4788,7 +4777,7 @@
         <v>6646.03</v>
       </c>
       <c r="I122">
-        <v>-0.24000000000069119</v>
+        <v>-0.2400000000006912</v>
       </c>
       <c r="J122" t="s">
         <v>214</v>
@@ -4820,7 +4809,7 @@
         <v>368.59</v>
       </c>
       <c r="I123">
-        <v>-0.24000000000000909</v>
+        <v>-0.2400000000000091</v>
       </c>
       <c r="J123" t="s">
         <v>214</v>
@@ -4849,10 +4838,10 @@
         <v>2452.04</v>
       </c>
       <c r="H124">
-        <v>2451.8000000000002</v>
+        <v>2451.8</v>
       </c>
       <c r="I124">
-        <v>-0.23999999999978169</v>
+        <v>-0.2399999999997817</v>
       </c>
       <c r="J124" t="s">
         <v>214</v>
@@ -4884,7 +4873,7 @@
         <v>13673.61</v>
       </c>
       <c r="I125">
-        <v>-0.23999999999978169</v>
+        <v>-0.2399999999997817</v>
       </c>
       <c r="J125" t="s">
         <v>214</v>
@@ -4904,10 +4893,10 @@
         <v>800</v>
       </c>
       <c r="E126">
-        <v>6793.0460000000003</v>
+        <v>6793.046</v>
       </c>
       <c r="F126">
-        <v>6793.0460000000003</v>
+        <v>6793.046</v>
       </c>
       <c r="G126">
         <v>202531.6</v>
@@ -4916,7 +4905,7 @@
         <v>202531.37</v>
       </c>
       <c r="I126">
-        <v>-0.23000000001047741</v>
+        <v>-0.2300000000104774</v>
       </c>
       <c r="J126" t="s">
         <v>214</v>
@@ -4942,13 +4931,13 @@
         <v>2220</v>
       </c>
       <c r="G127">
-        <v>19113.830000000002</v>
+        <v>19113.83</v>
       </c>
       <c r="H127">
-        <v>19113.599999999999</v>
+        <v>19113.6</v>
       </c>
       <c r="I127">
-        <v>-0.23000000000320139</v>
+        <v>-0.2300000000032014</v>
       </c>
       <c r="J127" t="s">
         <v>214</v>
@@ -4980,7 +4969,7 @@
         <v>496.46</v>
       </c>
       <c r="I128">
-        <v>-0.23000000000001819</v>
+        <v>-0.2300000000000182</v>
       </c>
       <c r="J128" t="s">
         <v>214</v>
@@ -5012,7 +5001,7 @@
         <v>2300.36</v>
       </c>
       <c r="I129">
-        <v>-0.23000000000001819</v>
+        <v>-0.2300000000000182</v>
       </c>
       <c r="J129" t="s">
         <v>214</v>
@@ -5044,7 +5033,7 @@
         <v>266489.02</v>
       </c>
       <c r="I130">
-        <v>-0.22999999998137349</v>
+        <v>-0.2299999999813735</v>
       </c>
       <c r="J130" t="s">
         <v>214</v>
@@ -5076,7 +5065,7 @@
         <v>6989.3</v>
       </c>
       <c r="I131">
-        <v>-0.22000000000025469</v>
+        <v>-0.2200000000002547</v>
       </c>
       <c r="J131" t="s">
         <v>214</v>
@@ -5108,7 +5097,7 @@
         <v>5405.31</v>
       </c>
       <c r="I132">
-        <v>-0.21999999999934519</v>
+        <v>-0.2199999999993452</v>
       </c>
       <c r="J132" t="s">
         <v>214</v>
@@ -5140,7 +5129,7 @@
         <v>15638.95</v>
       </c>
       <c r="I133">
-        <v>-0.20999999999912691</v>
+        <v>-0.2099999999991269</v>
       </c>
       <c r="J133" t="s">
         <v>214</v>
@@ -5172,7 +5161,7 @@
         <v>20570.93</v>
       </c>
       <c r="I134">
-        <v>-0.20999999999912691</v>
+        <v>-0.2099999999991269</v>
       </c>
       <c r="J134" t="s">
         <v>214</v>
@@ -5230,7 +5219,7 @@
         <v>4574</v>
       </c>
       <c r="G136">
-        <v>17793.060000000001</v>
+        <v>17793.06</v>
       </c>
       <c r="H136">
         <v>17792.86</v>
@@ -5288,19 +5277,19 @@
         <v>800</v>
       </c>
       <c r="E138">
-        <v>3024.2869999999998</v>
+        <v>3024.287</v>
       </c>
       <c r="F138">
-        <v>3024.2869999999998</v>
+        <v>3024.287</v>
       </c>
       <c r="G138">
-        <v>80137.149999999994</v>
+        <v>80137.14999999999</v>
       </c>
       <c r="H138">
         <v>80136.95</v>
       </c>
       <c r="I138">
-        <v>-0.19999999999708959</v>
+        <v>-0.1999999999970896</v>
       </c>
       <c r="J138" t="s">
         <v>214</v>
@@ -5326,13 +5315,13 @@
         <v>5241</v>
       </c>
       <c r="G139">
-        <v>20178.689999999999</v>
+        <v>20178.69</v>
       </c>
       <c r="H139">
-        <v>20178.490000000002</v>
+        <v>20178.49</v>
       </c>
       <c r="I139">
-        <v>-0.19999999999708959</v>
+        <v>-0.1999999999970896</v>
       </c>
       <c r="J139" t="s">
         <v>214</v>
@@ -5393,7 +5382,7 @@
         <v>2620.89</v>
       </c>
       <c r="H141">
-        <v>2620.6999999999998</v>
+        <v>2620.7</v>
       </c>
       <c r="I141">
         <v>-0.1900000000000546</v>
@@ -5416,10 +5405,10 @@
         <v>800</v>
       </c>
       <c r="E142">
-        <v>903.89599999999996</v>
+        <v>903.896</v>
       </c>
       <c r="F142">
-        <v>903.89599999999996</v>
+        <v>903.896</v>
       </c>
       <c r="G142">
         <v>7022.74</v>
@@ -5428,7 +5417,7 @@
         <v>7022.55</v>
       </c>
       <c r="I142">
-        <v>-0.18999999999959979</v>
+        <v>-0.1899999999995998</v>
       </c>
       <c r="J142" t="s">
         <v>214</v>
@@ -5454,10 +5443,10 @@
         <v>1338</v>
       </c>
       <c r="G143">
-        <v>9000.31</v>
+        <v>9000.309999999999</v>
       </c>
       <c r="H143">
-        <v>9000.1200000000008</v>
+        <v>9000.120000000001</v>
       </c>
       <c r="I143">
         <v>-0.1899999999986903</v>
@@ -5480,10 +5469,10 @@
         <v>800</v>
       </c>
       <c r="E144">
-        <v>730.89700000000005</v>
+        <v>730.897</v>
       </c>
       <c r="F144">
-        <v>730.89700000000005</v>
+        <v>730.897</v>
       </c>
       <c r="G144">
         <v>5101.84</v>
@@ -5492,7 +5481,7 @@
         <v>5101.66</v>
       </c>
       <c r="I144">
-        <v>-0.18000000000029101</v>
+        <v>-0.180000000000291</v>
       </c>
       <c r="J144" t="s">
         <v>214</v>
@@ -5518,13 +5507,13 @@
         <v>2694</v>
       </c>
       <c r="G145">
-        <v>17465.240000000002</v>
+        <v>17465.24</v>
       </c>
       <c r="H145">
-        <v>17465.060000000001</v>
+        <v>17465.06</v>
       </c>
       <c r="I145">
-        <v>-0.18000000000029101</v>
+        <v>-0.180000000000291</v>
       </c>
       <c r="J145" t="s">
         <v>214</v>
@@ -5556,7 +5545,7 @@
         <v>6932.59</v>
       </c>
       <c r="I146">
-        <v>-0.18000000000029101</v>
+        <v>-0.180000000000291</v>
       </c>
       <c r="J146" t="s">
         <v>214</v>
@@ -5576,10 +5565,10 @@
         <v>800</v>
       </c>
       <c r="E147">
-        <v>47.654000000000003</v>
+        <v>47.654</v>
       </c>
       <c r="F147">
-        <v>47.654000000000003</v>
+        <v>47.654</v>
       </c>
       <c r="G147">
         <v>2859.42</v>
@@ -5588,7 +5577,7 @@
         <v>2859.24</v>
       </c>
       <c r="I147">
-        <v>-0.18000000000029101</v>
+        <v>-0.180000000000291</v>
       </c>
       <c r="J147" t="s">
         <v>214</v>
@@ -5617,10 +5606,10 @@
         <v>9704.57</v>
       </c>
       <c r="H148">
-        <v>9704.39</v>
+        <v>9704.389999999999</v>
       </c>
       <c r="I148">
-        <v>-0.18000000000029101</v>
+        <v>-0.180000000000291</v>
       </c>
       <c r="J148" t="s">
         <v>214</v>
@@ -5652,7 +5641,7 @@
         <v>5787.99</v>
       </c>
       <c r="I149">
-        <v>-0.17000000000007279</v>
+        <v>-0.1700000000000728</v>
       </c>
       <c r="J149" t="s">
         <v>214</v>
@@ -5681,7 +5670,7 @@
         <v>37163.93</v>
       </c>
       <c r="H150">
-        <v>37163.760000000002</v>
+        <v>37163.76</v>
       </c>
       <c r="I150">
         <v>-0.1699999999982538</v>
@@ -5704,16 +5693,16 @@
         <v>800</v>
       </c>
       <c r="E151">
-        <v>1815.6030000000001</v>
+        <v>1815.603</v>
       </c>
       <c r="F151">
-        <v>1815.6030000000001</v>
+        <v>1815.603</v>
       </c>
       <c r="G151">
         <v>35082.47</v>
       </c>
       <c r="H151">
-        <v>35082.300000000003</v>
+        <v>35082.3</v>
       </c>
       <c r="I151">
         <v>-0.1699999999982538</v>
@@ -5736,19 +5725,19 @@
         <v>800</v>
       </c>
       <c r="E152">
-        <v>23419.532999999999</v>
+        <v>23419.533</v>
       </c>
       <c r="F152">
-        <v>23419.532999999999</v>
+        <v>23419.533</v>
       </c>
       <c r="G152">
-        <v>85327.82</v>
+        <v>85327.82000000001</v>
       </c>
       <c r="H152">
         <v>85327.66</v>
       </c>
       <c r="I152">
-        <v>-0.16000000000349249</v>
+        <v>-0.1600000000034925</v>
       </c>
       <c r="J152" t="s">
         <v>214</v>
@@ -5774,13 +5763,13 @@
         <v>357</v>
       </c>
       <c r="G153">
-        <v>1031.8900000000001</v>
+        <v>1031.89</v>
       </c>
       <c r="H153">
         <v>1031.73</v>
       </c>
       <c r="I153">
-        <v>-0.16000000000008191</v>
+        <v>-0.1600000000000819</v>
       </c>
       <c r="J153" t="s">
         <v>214</v>
@@ -5812,7 +5801,7 @@
         <v>1889.42</v>
       </c>
       <c r="I154">
-        <v>-0.15999999999985451</v>
+        <v>-0.1599999999998545</v>
       </c>
       <c r="J154" t="s">
         <v>214</v>
@@ -5838,13 +5827,13 @@
         <v>2835</v>
       </c>
       <c r="G155">
-        <v>8476.81</v>
+        <v>8476.809999999999</v>
       </c>
       <c r="H155">
         <v>8476.65</v>
       </c>
       <c r="I155">
-        <v>-0.15999999999985451</v>
+        <v>-0.1599999999998545</v>
       </c>
       <c r="J155" t="s">
         <v>214</v>
@@ -5876,7 +5865,7 @@
         <v>11168.91</v>
       </c>
       <c r="I156">
-        <v>-0.15999999999985451</v>
+        <v>-0.1599999999998545</v>
       </c>
       <c r="J156" t="s">
         <v>214</v>
@@ -5905,10 +5894,10 @@
         <v>2496.21</v>
       </c>
       <c r="H157">
-        <v>2496.0500000000002</v>
+        <v>2496.05</v>
       </c>
       <c r="I157">
-        <v>-0.15999999999985451</v>
+        <v>-0.1599999999998545</v>
       </c>
       <c r="J157" t="s">
         <v>214</v>
@@ -5928,19 +5917,19 @@
         <v>800</v>
       </c>
       <c r="E158">
-        <v>9584.3359999999993</v>
+        <v>9584.335999999999</v>
       </c>
       <c r="F158">
-        <v>9584.3359999999993</v>
+        <v>9584.335999999999</v>
       </c>
       <c r="G158">
-        <v>82575.179999999993</v>
+        <v>82575.17999999999</v>
       </c>
       <c r="H158">
         <v>82575.02</v>
       </c>
       <c r="I158">
-        <v>-0.15999999998894049</v>
+        <v>-0.1599999999889405</v>
       </c>
       <c r="J158" t="s">
         <v>214</v>
@@ -5960,19 +5949,19 @@
         <v>800</v>
       </c>
       <c r="E159">
-        <v>1213.8869999999999</v>
+        <v>1213.887</v>
       </c>
       <c r="F159">
-        <v>1213.8869999999999</v>
+        <v>1213.887</v>
       </c>
       <c r="G159">
         <v>27093.11</v>
       </c>
       <c r="H159">
-        <v>27092.959999999999</v>
+        <v>27092.96</v>
       </c>
       <c r="I159">
-        <v>-0.15000000000145519</v>
+        <v>-0.1500000000014552</v>
       </c>
       <c r="J159" t="s">
         <v>214</v>
@@ -6004,7 +5993,7 @@
         <v>21498.84</v>
       </c>
       <c r="I160">
-        <v>-0.15000000000145519</v>
+        <v>-0.1500000000014552</v>
       </c>
       <c r="J160" t="s">
         <v>214</v>
@@ -6036,7 +6025,7 @@
         <v>5350.11</v>
       </c>
       <c r="I161">
-        <v>-0.14000000000032739</v>
+        <v>-0.1400000000003274</v>
       </c>
       <c r="J161" t="s">
         <v>214</v>
@@ -6126,7 +6115,7 @@
         <v>5054</v>
       </c>
       <c r="G164">
-        <v>22488.639999999999</v>
+        <v>22488.64</v>
       </c>
       <c r="H164">
         <v>22488.5</v>
@@ -6196,7 +6185,7 @@
         <v>3920.27</v>
       </c>
       <c r="I166">
-        <v>-0.13000000000010911</v>
+        <v>-0.1300000000001091</v>
       </c>
       <c r="J166" t="s">
         <v>214</v>
@@ -6228,7 +6217,7 @@
         <v>3382.19</v>
       </c>
       <c r="I167">
-        <v>-0.13000000000010911</v>
+        <v>-0.1300000000001091</v>
       </c>
       <c r="J167" t="s">
         <v>214</v>
@@ -6248,10 +6237,10 @@
         <v>800</v>
       </c>
       <c r="E168">
-        <v>1321.1020000000001</v>
+        <v>1321.102</v>
       </c>
       <c r="F168">
-        <v>1321.1020000000001</v>
+        <v>1321.102</v>
       </c>
       <c r="G168">
         <v>16349.56</v>
@@ -6260,7 +6249,7 @@
         <v>16349.43</v>
       </c>
       <c r="I168">
-        <v>-0.12999999999919959</v>
+        <v>-0.1299999999991996</v>
       </c>
       <c r="J168" t="s">
         <v>214</v>
@@ -6388,7 +6377,7 @@
         <v>10681.36</v>
       </c>
       <c r="I172">
-        <v>-0.11999999999898139</v>
+        <v>-0.1199999999989814</v>
       </c>
       <c r="J172" t="s">
         <v>214</v>
@@ -6408,10 +6397,10 @@
         <v>800</v>
       </c>
       <c r="E173">
-        <v>792.40099999999995</v>
+        <v>792.401</v>
       </c>
       <c r="F173">
-        <v>792.40099999999995</v>
+        <v>792.401</v>
       </c>
       <c r="G173">
         <v>29979.93</v>
@@ -6420,7 +6409,7 @@
         <v>29979.81</v>
       </c>
       <c r="I173">
-        <v>-0.11999999999898139</v>
+        <v>-0.1199999999989814</v>
       </c>
       <c r="J173" t="s">
         <v>214</v>
@@ -6449,7 +6438,7 @@
         <v>37609.1</v>
       </c>
       <c r="H174">
-        <v>37608.980000000003</v>
+        <v>37608.98</v>
       </c>
       <c r="I174">
         <v>-0.1199999999953434</v>
@@ -6481,7 +6470,7 @@
         <v>4995.59</v>
       </c>
       <c r="H175">
-        <v>4995.4799999999996</v>
+        <v>4995.48</v>
       </c>
       <c r="I175">
         <v>-0.1100000000005821</v>
@@ -6504,10 +6493,10 @@
         <v>800</v>
       </c>
       <c r="E176">
-        <v>2842.3319999999999</v>
+        <v>2842.332</v>
       </c>
       <c r="F176">
-        <v>2842.3319999999999</v>
+        <v>2842.332</v>
       </c>
       <c r="G176">
         <v>108652.56</v>
@@ -6708,7 +6697,7 @@
         <v>6430.52</v>
       </c>
       <c r="I182">
-        <v>-9.9999999999454303E-2</v>
+        <v>-0.0999999999994543</v>
       </c>
       <c r="J182" t="s">
         <v>214</v>
@@ -6740,7 +6729,7 @@
         <v>31177.22</v>
       </c>
       <c r="I183">
-        <v>-9.9999999998544808E-2</v>
+        <v>-0.09999999999854481</v>
       </c>
       <c r="J183" t="s">
         <v>214</v>
@@ -6772,7 +6761,7 @@
         <v>7912.45</v>
       </c>
       <c r="I184">
-        <v>-9.0000000000145519E-2</v>
+        <v>-0.09000000000014552</v>
       </c>
       <c r="J184" t="s">
         <v>214</v>
@@ -6804,7 +6793,7 @@
         <v>1691.33</v>
       </c>
       <c r="I185">
-        <v>-9.0000000000145519E-2</v>
+        <v>-0.09000000000014552</v>
       </c>
       <c r="J185" t="s">
         <v>214</v>
@@ -6836,7 +6825,7 @@
         <v>80.27</v>
       </c>
       <c r="I186">
-        <v>-9.0000000000003411E-2</v>
+        <v>-0.09000000000000341</v>
       </c>
       <c r="J186" t="s">
         <v>214</v>
@@ -6868,7 +6857,7 @@
         <v>52.35</v>
       </c>
       <c r="I187">
-        <v>-8.9999999999996305E-2</v>
+        <v>-0.08999999999999631</v>
       </c>
       <c r="J187" t="s">
         <v>214</v>
@@ -6897,10 +6886,10 @@
         <v>32969.89</v>
       </c>
       <c r="H188">
-        <v>32969.800000000003</v>
+        <v>32969.8</v>
       </c>
       <c r="I188">
-        <v>-8.999999999650754E-2</v>
+        <v>-0.08999999999650754</v>
       </c>
       <c r="J188" t="s">
         <v>214</v>
@@ -6929,10 +6918,10 @@
         <v>31860</v>
       </c>
       <c r="H189">
-        <v>31859.919999999998</v>
+        <v>31859.92</v>
       </c>
       <c r="I189">
-        <v>-8.000000000174623E-2</v>
+        <v>-0.08000000000174623</v>
       </c>
       <c r="J189" t="s">
         <v>214</v>
@@ -6964,7 +6953,7 @@
         <v>44361.95</v>
       </c>
       <c r="I190">
-        <v>-8.000000000174623E-2</v>
+        <v>-0.08000000000174623</v>
       </c>
       <c r="J190" t="s">
         <v>214</v>
@@ -6996,7 +6985,7 @@
         <v>1758</v>
       </c>
       <c r="I191">
-        <v>-7.999999999992724E-2</v>
+        <v>-0.07999999999992724</v>
       </c>
       <c r="J191" t="s">
         <v>214</v>
@@ -7028,7 +7017,7 @@
         <v>2827.03</v>
       </c>
       <c r="I192">
-        <v>-7.999999999992724E-2</v>
+        <v>-0.07999999999992724</v>
       </c>
       <c r="J192" t="s">
         <v>214</v>
@@ -7060,7 +7049,7 @@
         <v>5420.97</v>
       </c>
       <c r="I193">
-        <v>-7.999999999992724E-2</v>
+        <v>-0.07999999999992724</v>
       </c>
       <c r="J193" t="s">
         <v>214</v>
@@ -7086,13 +7075,13 @@
         <v>22067</v>
       </c>
       <c r="G194">
-        <v>79096.789999999994</v>
+        <v>79096.78999999999</v>
       </c>
       <c r="H194">
-        <v>79096.710000000006</v>
+        <v>79096.71000000001</v>
       </c>
       <c r="I194">
-        <v>-7.9999999987194315E-2</v>
+        <v>-0.07999999998719431</v>
       </c>
       <c r="J194" t="s">
         <v>214</v>
@@ -7121,10 +7110,10 @@
         <v>9084.43</v>
       </c>
       <c r="H195">
-        <v>9084.36</v>
+        <v>9084.360000000001</v>
       </c>
       <c r="I195">
-        <v>-6.9999999999708962E-2</v>
+        <v>-0.06999999999970896</v>
       </c>
       <c r="J195" t="s">
         <v>214</v>
@@ -7156,7 +7145,7 @@
         <v>7784</v>
       </c>
       <c r="I196">
-        <v>-6.9999999999708962E-2</v>
+        <v>-0.06999999999970896</v>
       </c>
       <c r="J196" t="s">
         <v>214</v>
@@ -7188,7 +7177,7 @@
         <v>12098.26</v>
       </c>
       <c r="I197">
-        <v>-6.9999999999708962E-2</v>
+        <v>-0.06999999999970896</v>
       </c>
       <c r="J197" t="s">
         <v>214</v>
@@ -7214,13 +7203,13 @@
         <v>4391</v>
       </c>
       <c r="G198">
-        <v>8433.94</v>
+        <v>8433.940000000001</v>
       </c>
       <c r="H198">
-        <v>8433.89</v>
+        <v>8433.889999999999</v>
       </c>
       <c r="I198">
-        <v>-5.0000000001091387E-2</v>
+        <v>-0.05000000000109139</v>
       </c>
       <c r="J198" t="s">
         <v>214</v>
@@ -7252,7 +7241,7 @@
         <v>3763.27</v>
       </c>
       <c r="I199">
-        <v>-5.0000000000181899E-2</v>
+        <v>-0.0500000000001819</v>
       </c>
       <c r="J199" t="s">
         <v>214</v>
@@ -7281,10 +7270,10 @@
         <v>782.12</v>
       </c>
       <c r="H200">
-        <v>782.07</v>
+        <v>782.0700000000001</v>
       </c>
       <c r="I200">
-        <v>-4.9999999999954532E-2</v>
+        <v>-0.04999999999995453</v>
       </c>
       <c r="J200" t="s">
         <v>214</v>
@@ -7316,7 +7305,7 @@
         <v>7921.74</v>
       </c>
       <c r="I201">
-        <v>-3.999999999996362E-2</v>
+        <v>-0.03999999999996362</v>
       </c>
       <c r="J201" t="s">
         <v>214</v>

</xml_diff>